<commit_message>
Kompetenzmatrix: publish full-text v1.0 (issue #2)
Publish content/lehrkraefte/kompetenzmatrix (DE+EN) with the verified
full curriculum wording for all 27 competencies, grade/semester,
covered-by (P1-P5/Selbstlernen), and status. Corrects several grade
misassignments from the v0.1 draft (TB04, TB05, TB06, TB07, TB09,
TB02 Laufzeitabschaetzungen) and splits a previously merged TB11 row
into its two distinct competencies.

Source-verification detail moved to planning/KOMPETENZMATRIX-NOTES.md
(internal only). Backfill the corrected mapping into PLAN.md SS4,
bump to v1.0, and mark roadmap steps 1-2 done in SS7.

Ignore .DS_Store going forward.
</commit_message>
<xml_diff>
--- a/planning/LP-Informatik-Sek2-v1.3-nachBegutachtung.xlsx
+++ b/planning/LP-Informatik-Sek2-v1.3-nachBegutachtung.xlsx
@@ -6,8 +6,8 @@
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="9te-12teSchulstufe-2023" sheetId="1" state="hidden" r:id="rId2"/>
-    <sheet name="PF-NachBegutachtung-V1" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="9te-12teSchulstufe-2023" sheetId="1" state="hidden" r:id="rId3"/>
+    <sheet name="PF-NachBegutachtung-V1" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="460">
   <si>
     <t xml:space="preserve">Lehrplan Informatik Sek 2 - Zentrale Themenbereiche LP 9. 10. 11. 12</t>
   </si>
@@ -6487,6 +6487,9 @@
   </si>
   <si>
     <t xml:space="preserve">KI-Anwendungsbereiche vergleichen und begründen, welches Verfahren für einen gegebenen Problemtyp geeignet ist.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">04 Computersysteme</t>
   </si>
   <si>
     <t xml:space="preserve">Rechnersysteme (z.B. Einplatinenrechner oder virtuelle Maschinen), Peripherie und vernetzte Systeme</t>
@@ -7806,8 +7809,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Hörmann, Corinna (ext)" id="{85974B95-4007-0DDD-3354-E53A258B45AC}" userId="e1f560cd081541ba9763a674d14e2b6a@auth.local" providerId="Teamlab"/>
-  <person displayName="Bollin, Andreas" id="{19EA2D6B-4254-153B-433E-754A15D7A925}" userId="andreas.bollin@aau.at" providerId="Teamlab"/>
+  <person displayName="Hörmann, Corinna (ext)" id="{BFCBC2F8-A715-432B-5C14-0846DA503631}" userId="e1f560cd081541ba9763a674d14e2b6a@auth.local" providerId="Teamlab"/>
+  <person displayName="Bollin, Andreas" id="{5F4221FF-DB5C-582F-B93C-57CDE01E3627}" userId="andreas.bollin@aau.at" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -8303,31 +8306,31 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B18" dT="2026-09-01T16:25:40.14Z" personId="{85974B95-4007-0DDD-3354-E53A258B45AC}" id="{193CCF7B-8F84-35CF-F2A7-99B5E7C7D692}" done="0">
+  <threadedComment ref="B18" dT="2026-09-01T16:25:40.14Z" personId="{BFCBC2F8-A715-432B-5C14-0846DA503631}" id="{193CCF7B-8F84-35CF-F2A7-99B5E7C7D692}" done="0">
     <text xml:space="preserve">ich finde hier immer noch die Logik und Boolsche Algebra zu viel (aber ich weiß dass die ARGE das will)
 </text>
   </threadedComment>
-  <threadedComment ref="B18" dT="2026-09-02T12:03:19.79Z" personId="{19EA2D6B-4254-153B-433E-754A15D7A925}" id="{B2F05CA6-7853-B35E-D495-46E03724B41F}" parentId="{193CCF7B-8F84-35CF-F2A7-99B5E7C7D692}" done="0">
+  <threadedComment ref="B18" dT="2026-09-02T12:03:19.79Z" personId="{5F4221FF-DB5C-582F-B93C-57CDE01E3627}" id="{B2F05CA6-7853-B35E-D495-46E03724B41F}" parentId="{193CCF7B-8F84-35CF-F2A7-99B5E7C7D692}" done="0">
     <text xml:space="preserve">Na ja, ein wenig sollte das in DGB gemacht worden sein, ist halt Wiederholung.
 </text>
   </threadedComment>
-  <threadedComment ref="F19" dT="2026-09-01T16:24:47.67Z" personId="{85974B95-4007-0DDD-3354-E53A258B45AC}" id="{A17A6BA6-EAF0-0BA3-126C-861305FEE090}" done="1">
+  <threadedComment ref="F19" dT="2026-09-01T16:24:47.67Z" personId="{BFCBC2F8-A715-432B-5C14-0846DA503631}" id="{A17A6BA6-EAF0-0BA3-126C-861305FEE090}" done="1">
     <text xml:space="preserve">gegebene
 </text>
   </threadedComment>
-  <threadedComment ref="F19" dT="2026-09-02T12:03:59.86Z" personId="{19EA2D6B-4254-153B-433E-754A15D7A925}" id="{C6818490-4471-72D5-4517-24A794A9B605}" parentId="{A17A6BA6-EAF0-0BA3-126C-861305FEE090}" done="0">
+  <threadedComment ref="F19" dT="2026-09-02T12:03:59.86Z" personId="{5F4221FF-DB5C-582F-B93C-57CDE01E3627}" id="{C6818490-4471-72D5-4517-24A794A9B605}" parentId="{A17A6BA6-EAF0-0BA3-126C-861305FEE090}" done="0">
     <text xml:space="preserve">Danke. Korrigiert
 </text>
   </threadedComment>
-  <threadedComment ref="D78" dT="2026-09-01T16:32:16.80Z" personId="{85974B95-4007-0DDD-3354-E53A258B45AC}" id="{B2C8A4BF-9C12-6BFC-9D2E-69C3A644D679}" done="0">
+  <threadedComment ref="D78" dT="2026-09-01T16:32:16.80Z" personId="{BFCBC2F8-A715-432B-5C14-0846DA503631}" id="{B2C8A4BF-9C12-6BFC-9D2E-69C3A644D679}" done="0">
     <text xml:space="preserve">ich bin unschlüssig, ob wir den AI Act hier namentlich erwähnen sollen. Was wenn in 3 Jahren das Ding anders heißt? Ich wäre dafür, das als Beispiel in den did. Kommentar zu schreiben
 </text>
   </threadedComment>
-  <threadedComment ref="B80" dT="2026-09-01T16:32:53.96Z" personId="{85974B95-4007-0DDD-3354-E53A258B45AC}" id="{C8D77332-6942-7786-DCA2-E456E97BB1BD}" done="1">
+  <threadedComment ref="B80" dT="2026-09-01T16:32:53.96Z" personId="{BFCBC2F8-A715-432B-5C14-0846DA503631}" id="{C8D77332-6942-7786-DCA2-E456E97BB1BD}" done="1">
     <text xml:space="preserve">wie wäre es mit "(Berufs-)Alltag"?
 </text>
   </threadedComment>
-  <threadedComment ref="B80" dT="2026-09-02T11:22:54.76Z" personId="{19EA2D6B-4254-153B-433E-754A15D7A925}" id="{005CF391-EE7A-9761-BEA0-8FB54892FB86}" parentId="{C8D77332-6942-7786-DCA2-E456E97BB1BD}" done="0">
+  <threadedComment ref="B80" dT="2026-09-02T11:22:54.76Z" personId="{5F4221FF-DB5C-582F-B93C-57CDE01E3627}" id="{005CF391-EE7A-9761-BEA0-8FB54892FB86}" parentId="{C8D77332-6942-7786-DCA2-E456E97BB1BD}" done="0">
     <text xml:space="preserve">OK, Gute Idee
 </text>
   </threadedComment>
@@ -12915,10 +12918,12 @@
       <c r="R29" s="117"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="118"/>
-      <c r="B30" s="118"/>
-      <c r="C30" s="119"/>
-      <c r="D30" s="118"/>
+      <c r="A30" s="120" t="s">
+        <v>419</v>
+      </c>
+      <c r="B30" s="120"/>
+      <c r="C30" s="120"/>
+      <c r="D30" s="120"/>
       <c r="E30" s="119"/>
       <c r="F30" s="118"/>
       <c r="G30" s="119"/>
@@ -12967,7 +12972,7 @@
       <c r="B32" s="137"/>
       <c r="C32" s="112"/>
       <c r="D32" s="111" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E32" s="112"/>
       <c r="F32" s="110"/>
@@ -12991,7 +12996,7 @@
       <c r="B33" s="139"/>
       <c r="C33" s="115"/>
       <c r="D33" s="110" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E33" s="115" t="s">
         <v>44</v>
@@ -13061,7 +13066,7 @@
     </row>
     <row r="37" ht="18.75">
       <c r="A37" s="120" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B37" s="120"/>
       <c r="C37" s="120"/>
@@ -13132,13 +13137,13 @@
         <v>35</v>
       </c>
       <c r="B40" s="122" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="C40" s="112"/>
       <c r="D40" s="110"/>
       <c r="E40" s="115"/>
       <c r="F40" s="122" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G40" s="114"/>
     </row>
@@ -13147,7 +13152,7 @@
         <v>47</v>
       </c>
       <c r="B41" s="110" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C41" s="115" t="s">
         <v>401</v>
@@ -13155,7 +13160,7 @@
       <c r="D41" s="110"/>
       <c r="E41" s="115"/>
       <c r="F41" s="110" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="G41" s="115" t="s">
         <v>44</v>
@@ -13183,7 +13188,7 @@
     </row>
     <row r="43" ht="18.75">
       <c r="A43" s="120" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B43" s="120"/>
       <c r="C43" s="120"/>
@@ -13256,11 +13261,11 @@
       <c r="B46" s="110"/>
       <c r="C46" s="115"/>
       <c r="D46" s="122" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E46" s="112"/>
       <c r="F46" s="122" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G46" s="112"/>
     </row>
@@ -13271,13 +13276,13 @@
       <c r="B47" s="110"/>
       <c r="C47" s="115"/>
       <c r="D47" s="110" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E47" s="115" t="s">
         <v>44</v>
       </c>
       <c r="F47" s="110" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G47" s="115" t="s">
         <v>44</v>
@@ -13316,7 +13321,7 @@
     </row>
     <row r="49" ht="18.75">
       <c r="A49" s="120" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="B49" s="120"/>
       <c r="C49" s="120"/>
@@ -13389,7 +13394,7 @@
       <c r="B52" s="125"/>
       <c r="C52" s="112"/>
       <c r="D52" s="122" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E52" s="112"/>
       <c r="F52" s="125"/>
@@ -13402,7 +13407,7 @@
       <c r="B53" s="125"/>
       <c r="C53" s="115"/>
       <c r="D53" s="141" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E53" s="115" t="s">
         <v>37</v>
@@ -13443,7 +13448,7 @@
     </row>
     <row r="55" ht="18.75">
       <c r="A55" s="120" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B55" s="120"/>
       <c r="C55" s="120"/>
@@ -13514,15 +13519,15 @@
         <v>35</v>
       </c>
       <c r="B58" s="111" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="C58" s="112"/>
       <c r="D58" s="122" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E58" s="112"/>
       <c r="F58" s="122" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="G58" s="112"/>
     </row>
@@ -13531,19 +13536,19 @@
         <v>47</v>
       </c>
       <c r="B59" s="110" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="C59" s="115" t="s">
         <v>401</v>
       </c>
       <c r="D59" s="110" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="E59" s="115" t="s">
         <v>37</v>
       </c>
       <c r="F59" s="110" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G59" s="115" t="s">
         <v>37</v>
@@ -13571,7 +13576,7 @@
     </row>
     <row r="61" ht="18.75">
       <c r="A61" s="120" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B61" s="120"/>
       <c r="C61" s="120"/>
@@ -13642,7 +13647,7 @@
         <v>35</v>
       </c>
       <c r="B64" s="122" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="C64" s="112"/>
       <c r="D64" s="125"/>
@@ -13655,7 +13660,7 @@
         <v>47</v>
       </c>
       <c r="B65" s="110" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="C65" s="115" t="s">
         <v>401</v>
@@ -13707,7 +13712,7 @@
     </row>
     <row r="68" ht="18.75">
       <c r="A68" s="120" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B68" s="120"/>
       <c r="C68" s="120"/>
@@ -13778,15 +13783,15 @@
         <v>35</v>
       </c>
       <c r="B71" s="111" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C71" s="112"/>
       <c r="D71" s="122" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E71" s="112"/>
       <c r="F71" s="122" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G71" s="112"/>
     </row>
@@ -13795,19 +13800,19 @@
         <v>47</v>
       </c>
       <c r="B72" s="110" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C72" s="115" t="s">
         <v>401</v>
       </c>
       <c r="D72" s="110" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E72" s="115" t="s">
         <v>37</v>
       </c>
       <c r="F72" s="110" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="G72" s="115" t="s">
         <v>37</v>
@@ -13855,7 +13860,7 @@
     </row>
     <row r="75" ht="18.75">
       <c r="A75" s="120" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B75" s="120"/>
       <c r="C75" s="120"/>
@@ -13926,15 +13931,15 @@
         <v>35</v>
       </c>
       <c r="B78" s="122" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="C78" s="112"/>
       <c r="D78" s="111" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E78" s="112"/>
       <c r="F78" s="122" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G78" s="112"/>
     </row>
@@ -13943,19 +13948,19 @@
         <v>47</v>
       </c>
       <c r="B79" s="110" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C79" s="115" t="s">
         <v>401</v>
       </c>
       <c r="D79" s="110" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E79" s="115" t="s">
         <v>37</v>
       </c>
       <c r="F79" s="110" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G79" s="115" t="s">
         <v>44</v>
@@ -13966,7 +13971,7 @@
         <v>47</v>
       </c>
       <c r="B80" s="124" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="C80" s="129"/>
       <c r="D80" s="95"/>
@@ -14092,10 +14097,11 @@
       <c r="G99" s="97"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A30:D30"/>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="A49:D49"/>

</xml_diff>